<commit_message>
Planilha do Exterior: adiciona aba Dublin x planejamento
Compara as 28 urnas de saidas/dados.json com o Anexo I do TSE: 23 batem
(aptos dentro de 1-10 por urna) e 5 urnas (1.997 aptos) não constam do
Anexo I. Comparecimento de Dublin: piso 7.206, estimativa ~8.183 (premissa),
teto 9.203, contra 11.499 esperados no planejamento.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bzScsAppuh4phNPSzsByq
</commit_message>
<xml_diff>
--- a/saidas/exterior_2026_t1_comparecimento_por_municipio.xlsx
+++ b/saidas/exterior_2026_t1_comparecimento_por_municipio.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por município" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conferência" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dublin x planejamento" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conferência" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Por município'!$A$4:$H$169</definedName>
@@ -23,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,8 +47,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +67,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -97,6 +107,12 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5522,6 +5538,926 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="78" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dublin — resultado oficial (PDF TSE) x planejamento (saidas/dados.json), por urna</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cada urna = 1 seção principal + suas agregadas, contada uma vez. Linhas em vermelho: urna ausente do Anexo I do PDF (comparecimento desconhecido).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Urna (seção principal)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Aptos — planejamento (CSV)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Aptos — PDF</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Diferença de aptos</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Comparecimento — PDF</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>% comparecimento</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Situação</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3315</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>792</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>790</v>
+      </c>
+      <c r="D5" s="4">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>536</v>
+      </c>
+      <c r="F5" s="5">
+        <f>E5/C5</f>
+        <v/>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3322</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>794</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>792</v>
+      </c>
+      <c r="D6" s="4">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>503</v>
+      </c>
+      <c r="F6" s="5">
+        <f>E6/C6</f>
+        <v/>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3313</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>797</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>792</v>
+      </c>
+      <c r="D7" s="4">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>492</v>
+      </c>
+      <c r="F7" s="5">
+        <f>E7/C7</f>
+        <v/>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3311</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>630</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>626</v>
+      </c>
+      <c r="D8" s="4">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>384</v>
+      </c>
+      <c r="F8" s="5">
+        <f>E8/C8</f>
+        <v/>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3302</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>771</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>763</v>
+      </c>
+      <c r="D9" s="4">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>373</v>
+      </c>
+      <c r="F9" s="5">
+        <f>E9/C9</f>
+        <v/>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3179</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>676</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>670</v>
+      </c>
+      <c r="D10" s="4">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>349</v>
+      </c>
+      <c r="F10" s="5">
+        <f>E10/C10</f>
+        <v/>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>3306</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>766</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>761</v>
+      </c>
+      <c r="D11" s="4">
+        <f>C11-B11</f>
+        <v/>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>345</v>
+      </c>
+      <c r="F11" s="5">
+        <f>E11/C11</f>
+        <v/>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>3161</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>791</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>787</v>
+      </c>
+      <c r="D12" s="4">
+        <f>C12-B12</f>
+        <v/>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>328</v>
+      </c>
+      <c r="F12" s="5">
+        <f>E12/C12</f>
+        <v/>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>3245</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>781</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>778</v>
+      </c>
+      <c r="D13" s="4">
+        <f>C13-B13</f>
+        <v/>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>322</v>
+      </c>
+      <c r="F13" s="5">
+        <f>E13/C13</f>
+        <v/>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3108</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>756</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>752</v>
+      </c>
+      <c r="D14" s="4">
+        <f>C14-B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>320</v>
+      </c>
+      <c r="F14" s="5">
+        <f>E14/C14</f>
+        <v/>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>3142</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>793</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>787</v>
+      </c>
+      <c r="D15" s="4">
+        <f>C15-B15</f>
+        <v/>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>318</v>
+      </c>
+      <c r="F15" s="5">
+        <f>E15/C15</f>
+        <v/>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>3229</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>606</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>601</v>
+      </c>
+      <c r="D16" s="4">
+        <f>C16-B16</f>
+        <v/>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>318</v>
+      </c>
+      <c r="F16" s="5">
+        <f>E16/C16</f>
+        <v/>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>3309</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>615</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>614</v>
+      </c>
+      <c r="D17" s="4">
+        <f>C17-B17</f>
+        <v/>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>278</v>
+      </c>
+      <c r="F17" s="5">
+        <f>E17/C17</f>
+        <v/>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>3216</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>571</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>568</v>
+      </c>
+      <c r="D18" s="4">
+        <f>C18-B18</f>
+        <v/>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>278</v>
+      </c>
+      <c r="F18" s="5">
+        <f>E18/C18</f>
+        <v/>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>3305</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>767</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>764</v>
+      </c>
+      <c r="D19" s="4">
+        <f>C19-B19</f>
+        <v/>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>265</v>
+      </c>
+      <c r="F19" s="5">
+        <f>E19/C19</f>
+        <v/>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>3078</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>429</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>427</v>
+      </c>
+      <c r="D20" s="4">
+        <f>C20-B20</f>
+        <v/>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>259</v>
+      </c>
+      <c r="F20" s="5">
+        <f>E20/C20</f>
+        <v/>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>3054</v>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>454</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>452</v>
+      </c>
+      <c r="D21" s="4">
+        <f>C21-B21</f>
+        <v/>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>256</v>
+      </c>
+      <c r="F21" s="5">
+        <f>E21/C21</f>
+        <v/>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1160</v>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>473</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>472</v>
+      </c>
+      <c r="D22" s="4">
+        <f>C22-B22</f>
+        <v/>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>239</v>
+      </c>
+      <c r="F22" s="5">
+        <f>E22/C22</f>
+        <v/>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>511</v>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>582</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>582</v>
+      </c>
+      <c r="D23" s="4">
+        <f>C23-B23</f>
+        <v/>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>226</v>
+      </c>
+      <c r="F23" s="5">
+        <f>E23/C23</f>
+        <v/>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>517</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>513</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>512</v>
+      </c>
+      <c r="D24" s="4">
+        <f>C24-B24</f>
+        <v/>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="F24" s="5">
+        <f>E24/C24</f>
+        <v/>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>512</v>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>476</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>476</v>
+      </c>
+      <c r="D25" s="4">
+        <f>C25-B25</f>
+        <v/>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>204</v>
+      </c>
+      <c r="F25" s="5">
+        <f>E25/C25</f>
+        <v/>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1352</v>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>462</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>462</v>
+      </c>
+      <c r="D26" s="4">
+        <f>C26-B26</f>
+        <v/>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>203</v>
+      </c>
+      <c r="F26" s="5">
+        <f>E26/C26</f>
+        <v/>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>513</v>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>502</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>501</v>
+      </c>
+      <c r="D27" s="4">
+        <f>C27-B27</f>
+        <v/>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>190</v>
+      </c>
+      <c r="F27" s="5">
+        <f>E27/C27</f>
+        <v/>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>no PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="n">
+        <v>3688</v>
+      </c>
+      <c r="B28" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="16" t="n"/>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>AUSENTE do Anexo I</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="n">
+        <v>3862</v>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="16" t="n"/>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>AUSENTE do Anexo I</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="n">
+        <v>3832</v>
+      </c>
+      <c r="B30" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="C30" s="15" t="n"/>
+      <c r="D30" s="15" t="n"/>
+      <c r="E30" s="15" t="n"/>
+      <c r="F30" s="16" t="n"/>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>AUSENTE do Anexo I</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="n">
+        <v>3308</v>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>399</v>
+      </c>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="15" t="n"/>
+      <c r="F31" s="16" t="n"/>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>AUSENTE do Anexo I</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="n">
+        <v>3442</v>
+      </c>
+      <c r="B32" s="15" t="n">
+        <v>398</v>
+      </c>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="16" t="n"/>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>AUSENTE do Anexo I</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B33" s="17">
+        <f>SUM(B5:B32)</f>
+        <v/>
+      </c>
+      <c r="C33" s="17">
+        <f>SUM(C5:C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="17">
+        <f>SUM(D5:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="17">
+        <f>SUM(E5:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="18">
+        <f>E33/C33</f>
+        <v/>
+      </c>
+      <c r="G33" s="13" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>Comparecimento total de Dublin — faixa</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Planejamento: comparecimento esperado (base B, prancheta Paredes_ABC)</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>11499</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Aptos nas urnas ausentes (planejamento)</t>
+        </is>
+      </c>
+      <c r="B37" s="4">
+        <f>SUMIF(G5:G32,"AUSENTE do Anexo I",B5:B32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Piso: só o que está no PDF</t>
+        </is>
+      </c>
+      <c r="B38" s="4">
+        <f>E33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Premissa: % de comparecimento das urnas ausentes (hipótese = taxa das 23 urnas do PDF; editável)</t>
+        </is>
+      </c>
+      <c r="B39" s="8">
+        <f>F33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Estimativa central de Dublin</t>
+        </is>
+      </c>
+      <c r="B40" s="4">
+        <f>E33+B37*B39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Teto: se as urnas ausentes tivessem 100% de comparecimento</t>
+        </is>
+      </c>
+      <c r="B41" s="4">
+        <f>E33+B37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Queda frente ao planejamento — piso (%)</t>
+        </is>
+      </c>
+      <c r="B42" s="5">
+        <f>B38/B36-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Queda frente ao planejamento — estimativa central (%)</t>
+        </is>
+      </c>
+      <c r="B43" s="5">
+        <f>B40/B36-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Queda frente ao planejamento — teto (%)</t>
+        </is>
+      </c>
+      <c r="B44" s="5">
+        <f>B41/B36-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>A estimativa central é premissa, não dado: o comparecimento real das 5 urnas ausentes só sai do CSV/Resultados do TSE.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5634,7 +6570,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Planilha do Exterior: corrige Dublin com os números do portal TSE
Conferidos 1:1 com o portal: Genebra, Frankfurt, Edimburgo e Ciudad del Este
(exatos) e Dublin, que no Anexo I omitia 5 urnas. Dublin: 28 seções, 16.720
aptos, comparecimento 8.417 (50,3%), 26,8% abaixo dos 11.499 do planejamento.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bzScsAppuh4phNPSzsByq
</commit_message>
<xml_diff>
--- a/saidas/exterior_2026_t1_comparecimento_por_municipio.xlsx
+++ b/saidas/exterior_2026_t1_comparecimento_por_municipio.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Por município'!$A$4:$H$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Por município'!$A$4:$I$169</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H170"/>
+  <dimension ref="A1:I170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -489,6 +489,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,7 +502,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fonte: TSE, Relatório Resultado da Totalização (SISTOT), Anexo I. ATENÇÃO: o anexo lista só seções com registro de ocorrência; os valores por município são, portanto, piso (ver aba "Conferência").</t>
+          <t>Fonte: TSE, Relatório Resultado da Totalização (SISTOT), Anexo I. ATENÇÃO: o anexo lista só seções com registro de ocorrência; salvo onde a coluna I indica o portal, os valores são piso (ver aba "Conferência").</t>
         </is>
       </c>
     </row>
@@ -546,6 +547,11 @@
           <t>% comparecimento</t>
         </is>
       </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Fonte / conferência</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -575,6 +581,11 @@
       <c r="H5" s="5">
         <f>IF(E5=0,0,F5/E5)</f>
         <v/>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -606,6 +617,11 @@
         <f>IF(E6=0,0,F6/E6)</f>
         <v/>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -636,6 +652,11 @@
         <f>IF(E7=0,0,F7/E7)</f>
         <v/>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -666,6 +687,11 @@
         <f>IF(E8=0,0,F8/E8)</f>
         <v/>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -696,6 +722,11 @@
         <f>IF(E9=0,0,F9/E9)</f>
         <v/>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -726,6 +757,11 @@
         <f>IF(E10=0,0,F10/E10)</f>
         <v/>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -756,6 +792,11 @@
         <f>IF(E11=0,0,F11/E11)</f>
         <v/>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -786,6 +827,11 @@
         <f>IF(E12=0,0,F12/E12)</f>
         <v/>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -816,6 +862,11 @@
         <f>IF(E13=0,0,F13/E13)</f>
         <v/>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -846,6 +897,11 @@
         <f>IF(E14=0,0,F14/E14)</f>
         <v/>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -876,35 +932,45 @@
         <f>IF(E15=0,0,F15/E15)</f>
         <v/>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B16" t="n">
-        <v>29386</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>BERLIM</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>15066</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>8204</v>
-      </c>
-      <c r="G16" s="4">
+      <c r="B16" s="6" t="n">
+        <v>29661</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>DUBLIN</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>16720</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>8417</v>
+      </c>
+      <c r="G16" s="7">
         <f>E16-F16</f>
         <v/>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="8">
         <f>IF(E16=0,0,F16/E16)</f>
         <v/>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Portal TSE (captura 07/10/2026) — substitui o Anexo I, que omitia 5 urnas</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -912,21 +978,21 @@
         <v>13</v>
       </c>
       <c r="B17" t="n">
-        <v>30120</v>
+        <v>29386</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MILÃO</t>
+          <t>BERLIM</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>24594</v>
+        <v>15066</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>7455</v>
+        <v>8204</v>
       </c>
       <c r="G17" s="4">
         <f>E17-F17</f>
@@ -936,35 +1002,45 @@
         <f>IF(E17=0,0,F17/E17)</f>
         <v/>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n">
+      <c r="A18" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="6" t="n">
-        <v>29661</v>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>DUBLIN</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="E18" s="7" t="n">
-        <v>14729</v>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>7206</v>
-      </c>
-      <c r="G18" s="7">
+      <c r="B18" t="n">
+        <v>30120</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MILÃO</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>24594</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>7455</v>
+      </c>
+      <c r="G18" s="4">
         <f>E18-F18</f>
         <v/>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="5">
         <f>IF(E18=0,0,F18/E18)</f>
         <v/>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -996,6 +1072,11 @@
         <f>IF(E19=0,0,F19/E19)</f>
         <v/>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1026,6 +1107,11 @@
         <f>IF(E20=0,0,F20/E20)</f>
         <v/>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1056,6 +1142,11 @@
         <f>IF(E21=0,0,F21/E21)</f>
         <v/>
       </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1086,6 +1177,11 @@
         <f>IF(E22=0,0,F22/E22)</f>
         <v/>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1116,6 +1212,11 @@
         <f>IF(E23=0,0,F23/E23)</f>
         <v/>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1146,6 +1247,11 @@
         <f>IF(E24=0,0,F24/E24)</f>
         <v/>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1176,6 +1282,11 @@
         <f>IF(E25=0,0,F25/E25)</f>
         <v/>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Anexo I; confere com o portal</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1206,6 +1317,11 @@
         <f>IF(E26=0,0,F26/E26)</f>
         <v/>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1236,6 +1352,11 @@
         <f>IF(E27=0,0,F27/E27)</f>
         <v/>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1266,6 +1387,11 @@
         <f>IF(E28=0,0,F28/E28)</f>
         <v/>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1296,6 +1422,11 @@
         <f>IF(E29=0,0,F29/E29)</f>
         <v/>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Anexo I; confere com o portal</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1326,6 +1457,11 @@
         <f>IF(E30=0,0,F30/E30)</f>
         <v/>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1356,6 +1492,11 @@
         <f>IF(E31=0,0,F31/E31)</f>
         <v/>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1386,6 +1527,11 @@
         <f>IF(E32=0,0,F32/E32)</f>
         <v/>
       </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1416,6 +1562,11 @@
         <f>IF(E33=0,0,F33/E33)</f>
         <v/>
       </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1446,6 +1597,11 @@
         <f>IF(E34=0,0,F34/E34)</f>
         <v/>
       </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1476,6 +1632,11 @@
         <f>IF(E35=0,0,F35/E35)</f>
         <v/>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1506,6 +1667,11 @@
         <f>IF(E36=0,0,F36/E36)</f>
         <v/>
       </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1536,6 +1702,11 @@
         <f>IF(E37=0,0,F37/E37)</f>
         <v/>
       </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1566,6 +1737,11 @@
         <f>IF(E38=0,0,F38/E38)</f>
         <v/>
       </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1596,6 +1772,11 @@
         <f>IF(E39=0,0,F39/E39)</f>
         <v/>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1626,6 +1807,11 @@
         <f>IF(E40=0,0,F40/E40)</f>
         <v/>
       </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Anexo I; confere com o portal</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1656,6 +1842,11 @@
         <f>IF(E41=0,0,F41/E41)</f>
         <v/>
       </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1686,6 +1877,11 @@
         <f>IF(E42=0,0,F42/E42)</f>
         <v/>
       </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1716,6 +1912,11 @@
         <f>IF(E43=0,0,F43/E43)</f>
         <v/>
       </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1746,6 +1947,11 @@
         <f>IF(E44=0,0,F44/E44)</f>
         <v/>
       </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1776,6 +1982,11 @@
         <f>IF(E45=0,0,F45/E45)</f>
         <v/>
       </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1806,6 +2017,11 @@
         <f>IF(E46=0,0,F46/E46)</f>
         <v/>
       </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1836,6 +2052,11 @@
         <f>IF(E47=0,0,F47/E47)</f>
         <v/>
       </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1866,6 +2087,11 @@
         <f>IF(E48=0,0,F48/E48)</f>
         <v/>
       </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1896,6 +2122,11 @@
         <f>IF(E49=0,0,F49/E49)</f>
         <v/>
       </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1926,6 +2157,11 @@
         <f>IF(E50=0,0,F50/E50)</f>
         <v/>
       </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1956,6 +2192,11 @@
         <f>IF(E51=0,0,F51/E51)</f>
         <v/>
       </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1986,6 +2227,11 @@
         <f>IF(E52=0,0,F52/E52)</f>
         <v/>
       </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2016,6 +2262,11 @@
         <f>IF(E53=0,0,F53/E53)</f>
         <v/>
       </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2046,6 +2297,11 @@
         <f>IF(E54=0,0,F54/E54)</f>
         <v/>
       </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2076,6 +2332,11 @@
         <f>IF(E55=0,0,F55/E55)</f>
         <v/>
       </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2106,6 +2367,11 @@
         <f>IF(E56=0,0,F56/E56)</f>
         <v/>
       </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2136,6 +2402,11 @@
         <f>IF(E57=0,0,F57/E57)</f>
         <v/>
       </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2166,6 +2437,11 @@
         <f>IF(E58=0,0,F58/E58)</f>
         <v/>
       </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2196,6 +2472,11 @@
         <f>IF(E59=0,0,F59/E59)</f>
         <v/>
       </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2226,6 +2507,11 @@
         <f>IF(E60=0,0,F60/E60)</f>
         <v/>
       </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Anexo I; confere com o portal</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2256,6 +2542,11 @@
         <f>IF(E61=0,0,F61/E61)</f>
         <v/>
       </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2286,6 +2577,11 @@
         <f>IF(E62=0,0,F62/E62)</f>
         <v/>
       </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2316,6 +2612,11 @@
         <f>IF(E63=0,0,F63/E63)</f>
         <v/>
       </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2346,6 +2647,11 @@
         <f>IF(E64=0,0,F64/E64)</f>
         <v/>
       </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2376,6 +2682,11 @@
         <f>IF(E65=0,0,F65/E65)</f>
         <v/>
       </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2406,6 +2717,11 @@
         <f>IF(E66=0,0,F66/E66)</f>
         <v/>
       </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2436,6 +2752,11 @@
         <f>IF(E67=0,0,F67/E67)</f>
         <v/>
       </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2466,6 +2787,11 @@
         <f>IF(E68=0,0,F68/E68)</f>
         <v/>
       </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2496,6 +2822,11 @@
         <f>IF(E69=0,0,F69/E69)</f>
         <v/>
       </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2526,6 +2857,11 @@
         <f>IF(E70=0,0,F70/E70)</f>
         <v/>
       </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2556,6 +2892,11 @@
         <f>IF(E71=0,0,F71/E71)</f>
         <v/>
       </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2586,6 +2927,11 @@
         <f>IF(E72=0,0,F72/E72)</f>
         <v/>
       </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2616,6 +2962,11 @@
         <f>IF(E73=0,0,F73/E73)</f>
         <v/>
       </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2646,6 +2997,11 @@
         <f>IF(E74=0,0,F74/E74)</f>
         <v/>
       </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2676,6 +3032,11 @@
         <f>IF(E75=0,0,F75/E75)</f>
         <v/>
       </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2706,6 +3067,11 @@
         <f>IF(E76=0,0,F76/E76)</f>
         <v/>
       </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2736,6 +3102,11 @@
         <f>IF(E77=0,0,F77/E77)</f>
         <v/>
       </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2766,6 +3137,11 @@
         <f>IF(E78=0,0,F78/E78)</f>
         <v/>
       </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2796,6 +3172,11 @@
         <f>IF(E79=0,0,F79/E79)</f>
         <v/>
       </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2826,6 +3207,11 @@
         <f>IF(E80=0,0,F80/E80)</f>
         <v/>
       </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2856,6 +3242,11 @@
         <f>IF(E81=0,0,F81/E81)</f>
         <v/>
       </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2886,6 +3277,11 @@
         <f>IF(E82=0,0,F82/E82)</f>
         <v/>
       </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2916,6 +3312,11 @@
         <f>IF(E83=0,0,F83/E83)</f>
         <v/>
       </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2946,6 +3347,11 @@
         <f>IF(E84=0,0,F84/E84)</f>
         <v/>
       </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2976,6 +3382,11 @@
         <f>IF(E85=0,0,F85/E85)</f>
         <v/>
       </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3006,6 +3417,11 @@
         <f>IF(E86=0,0,F86/E86)</f>
         <v/>
       </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -3036,6 +3452,11 @@
         <f>IF(E87=0,0,F87/E87)</f>
         <v/>
       </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -3066,6 +3487,11 @@
         <f>IF(E88=0,0,F88/E88)</f>
         <v/>
       </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -3096,6 +3522,11 @@
         <f>IF(E89=0,0,F89/E89)</f>
         <v/>
       </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -3126,6 +3557,11 @@
         <f>IF(E90=0,0,F90/E90)</f>
         <v/>
       </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -3156,6 +3592,11 @@
         <f>IF(E91=0,0,F91/E91)</f>
         <v/>
       </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -3186,6 +3627,11 @@
         <f>IF(E92=0,0,F92/E92)</f>
         <v/>
       </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3216,6 +3662,11 @@
         <f>IF(E93=0,0,F93/E93)</f>
         <v/>
       </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3246,6 +3697,11 @@
         <f>IF(E94=0,0,F94/E94)</f>
         <v/>
       </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -3276,6 +3732,11 @@
         <f>IF(E95=0,0,F95/E95)</f>
         <v/>
       </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -3306,6 +3767,11 @@
         <f>IF(E96=0,0,F96/E96)</f>
         <v/>
       </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -3336,6 +3802,11 @@
         <f>IF(E97=0,0,F97/E97)</f>
         <v/>
       </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -3366,6 +3837,11 @@
         <f>IF(E98=0,0,F98/E98)</f>
         <v/>
       </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -3396,6 +3872,11 @@
         <f>IF(E99=0,0,F99/E99)</f>
         <v/>
       </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -3426,6 +3907,11 @@
         <f>IF(E100=0,0,F100/E100)</f>
         <v/>
       </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -3456,6 +3942,11 @@
         <f>IF(E101=0,0,F101/E101)</f>
         <v/>
       </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -3486,6 +3977,11 @@
         <f>IF(E102=0,0,F102/E102)</f>
         <v/>
       </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -3516,6 +4012,11 @@
         <f>IF(E103=0,0,F103/E103)</f>
         <v/>
       </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -3546,6 +4047,11 @@
         <f>IF(E104=0,0,F104/E104)</f>
         <v/>
       </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -3576,6 +4082,11 @@
         <f>IF(E105=0,0,F105/E105)</f>
         <v/>
       </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -3606,6 +4117,11 @@
         <f>IF(E106=0,0,F106/E106)</f>
         <v/>
       </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -3636,6 +4152,11 @@
         <f>IF(E107=0,0,F107/E107)</f>
         <v/>
       </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -3666,6 +4187,11 @@
         <f>IF(E108=0,0,F108/E108)</f>
         <v/>
       </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -3696,6 +4222,11 @@
         <f>IF(E109=0,0,F109/E109)</f>
         <v/>
       </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -3726,6 +4257,11 @@
         <f>IF(E110=0,0,F110/E110)</f>
         <v/>
       </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -3756,6 +4292,11 @@
         <f>IF(E111=0,0,F111/E111)</f>
         <v/>
       </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -3786,6 +4327,11 @@
         <f>IF(E112=0,0,F112/E112)</f>
         <v/>
       </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -3816,6 +4362,11 @@
         <f>IF(E113=0,0,F113/E113)</f>
         <v/>
       </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -3846,6 +4397,11 @@
         <f>IF(E114=0,0,F114/E114)</f>
         <v/>
       </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -3876,6 +4432,11 @@
         <f>IF(E115=0,0,F115/E115)</f>
         <v/>
       </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -3906,6 +4467,11 @@
         <f>IF(E116=0,0,F116/E116)</f>
         <v/>
       </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -3936,6 +4502,11 @@
         <f>IF(E117=0,0,F117/E117)</f>
         <v/>
       </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -3966,6 +4537,11 @@
         <f>IF(E118=0,0,F118/E118)</f>
         <v/>
       </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -3996,6 +4572,11 @@
         <f>IF(E119=0,0,F119/E119)</f>
         <v/>
       </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -4026,6 +4607,11 @@
         <f>IF(E120=0,0,F120/E120)</f>
         <v/>
       </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -4056,6 +4642,11 @@
         <f>IF(E121=0,0,F121/E121)</f>
         <v/>
       </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -4086,6 +4677,11 @@
         <f>IF(E122=0,0,F122/E122)</f>
         <v/>
       </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -4116,6 +4712,11 @@
         <f>IF(E123=0,0,F123/E123)</f>
         <v/>
       </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -4146,6 +4747,11 @@
         <f>IF(E124=0,0,F124/E124)</f>
         <v/>
       </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -4176,6 +4782,11 @@
         <f>IF(E125=0,0,F125/E125)</f>
         <v/>
       </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -4206,6 +4817,11 @@
         <f>IF(E126=0,0,F126/E126)</f>
         <v/>
       </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -4236,6 +4852,11 @@
         <f>IF(E127=0,0,F127/E127)</f>
         <v/>
       </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -4266,6 +4887,11 @@
         <f>IF(E128=0,0,F128/E128)</f>
         <v/>
       </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -4296,6 +4922,11 @@
         <f>IF(E129=0,0,F129/E129)</f>
         <v/>
       </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -4326,6 +4957,11 @@
         <f>IF(E130=0,0,F130/E130)</f>
         <v/>
       </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -4356,6 +4992,11 @@
         <f>IF(E131=0,0,F131/E131)</f>
         <v/>
       </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -4386,6 +5027,11 @@
         <f>IF(E132=0,0,F132/E132)</f>
         <v/>
       </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -4416,6 +5062,11 @@
         <f>IF(E133=0,0,F133/E133)</f>
         <v/>
       </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -4446,6 +5097,11 @@
         <f>IF(E134=0,0,F134/E134)</f>
         <v/>
       </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -4476,6 +5132,11 @@
         <f>IF(E135=0,0,F135/E135)</f>
         <v/>
       </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -4506,6 +5167,11 @@
         <f>IF(E136=0,0,F136/E136)</f>
         <v/>
       </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -4536,6 +5202,11 @@
         <f>IF(E137=0,0,F137/E137)</f>
         <v/>
       </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -4566,6 +5237,11 @@
         <f>IF(E138=0,0,F138/E138)</f>
         <v/>
       </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -4596,6 +5272,11 @@
         <f>IF(E139=0,0,F139/E139)</f>
         <v/>
       </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -4626,6 +5307,11 @@
         <f>IF(E140=0,0,F140/E140)</f>
         <v/>
       </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -4656,6 +5342,11 @@
         <f>IF(E141=0,0,F141/E141)</f>
         <v/>
       </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -4686,6 +5377,11 @@
         <f>IF(E142=0,0,F142/E142)</f>
         <v/>
       </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -4716,6 +5412,11 @@
         <f>IF(E143=0,0,F143/E143)</f>
         <v/>
       </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -4746,6 +5447,11 @@
         <f>IF(E144=0,0,F144/E144)</f>
         <v/>
       </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -4776,6 +5482,11 @@
         <f>IF(E145=0,0,F145/E145)</f>
         <v/>
       </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -4806,6 +5517,11 @@
         <f>IF(E146=0,0,F146/E146)</f>
         <v/>
       </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -4836,6 +5552,11 @@
         <f>IF(E147=0,0,F147/E147)</f>
         <v/>
       </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -4866,6 +5587,11 @@
         <f>IF(E148=0,0,F148/E148)</f>
         <v/>
       </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -4896,6 +5622,11 @@
         <f>IF(E149=0,0,F149/E149)</f>
         <v/>
       </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -4926,6 +5657,11 @@
         <f>IF(E150=0,0,F150/E150)</f>
         <v/>
       </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -4956,6 +5692,11 @@
         <f>IF(E151=0,0,F151/E151)</f>
         <v/>
       </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -4986,6 +5727,11 @@
         <f>IF(E152=0,0,F152/E152)</f>
         <v/>
       </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -5016,6 +5762,11 @@
         <f>IF(E153=0,0,F153/E153)</f>
         <v/>
       </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -5046,6 +5797,11 @@
         <f>IF(E154=0,0,F154/E154)</f>
         <v/>
       </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -5076,6 +5832,11 @@
         <f>IF(E155=0,0,F155/E155)</f>
         <v/>
       </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -5106,6 +5867,11 @@
         <f>IF(E156=0,0,F156/E156)</f>
         <v/>
       </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -5136,6 +5902,11 @@
         <f>IF(E157=0,0,F157/E157)</f>
         <v/>
       </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -5166,6 +5937,11 @@
         <f>IF(E158=0,0,F158/E158)</f>
         <v/>
       </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -5196,6 +5972,11 @@
         <f>IF(E159=0,0,F159/E159)</f>
         <v/>
       </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -5226,6 +6007,11 @@
         <f>IF(E160=0,0,F160/E160)</f>
         <v/>
       </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -5256,6 +6042,11 @@
         <f>IF(E161=0,0,F161/E161)</f>
         <v/>
       </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -5286,6 +6077,11 @@
         <f>IF(E162=0,0,F162/E162)</f>
         <v/>
       </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -5316,6 +6112,11 @@
         <f>IF(E163=0,0,F163/E163)</f>
         <v/>
       </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -5346,6 +6147,11 @@
         <f>IF(E164=0,0,F164/E164)</f>
         <v/>
       </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -5376,6 +6182,11 @@
         <f>IF(E165=0,0,F165/E165)</f>
         <v/>
       </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -5406,6 +6217,11 @@
         <f>IF(E166=0,0,F166/E166)</f>
         <v/>
       </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -5436,6 +6252,11 @@
         <f>IF(E167=0,0,F167/E167)</f>
         <v/>
       </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -5466,6 +6287,11 @@
         <f>IF(E168=0,0,F168/E168)</f>
         <v/>
       </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -5495,6 +6321,11 @@
       <c r="H169" s="5">
         <f>IF(E169=0,0,F169/E169)</f>
         <v/>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Anexo I (piso)</t>
+        </is>
       </c>
     </row>
     <row r="170">
@@ -5502,7 +6333,7 @@
       <c r="B170" s="9" t="n"/>
       <c r="C170" s="9" t="inlineStr">
         <is>
-          <t>Soma dos municípios (Anexo I)</t>
+          <t>Soma dos municípios</t>
         </is>
       </c>
       <c r="D170" s="10">
@@ -5527,7 +6358,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H169"/>
+  <autoFilter ref="A4:I169"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5538,7 +6369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -6338,7 +7169,7 @@
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>Comparecimento total de Dublin — faixa</t>
+          <t>Comparecimento total de Dublin — oficial x planejamento</t>
         </is>
       </c>
     </row>
@@ -6355,95 +7186,104 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Aptos nas urnas ausentes (planejamento)</t>
-        </is>
-      </c>
-      <c r="B37" s="4">
-        <f>SUMIF(G5:G32,"AUSENTE do Anexo I",B5:B32)</f>
-        <v/>
+          <t>Resultado oficial — portal TSE (captura 07/10/2026): comparecimento</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>8417</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Piso: só o que está no PDF</t>
-        </is>
-      </c>
-      <c r="B38" s="4">
-        <f>E33</f>
+          <t>Queda frente ao planejamento (%)</t>
+        </is>
+      </c>
+      <c r="B38" s="5">
+        <f>B37/B36-1</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Premissa: % de comparecimento das urnas ausentes (hipótese = taxa das 23 urnas do PDF; editável)</t>
-        </is>
-      </c>
-      <c r="B39" s="8">
-        <f>F33</f>
+          <t>Queda frente ao planejamento (eleitores)</t>
+        </is>
+      </c>
+      <c r="B39" s="4">
+        <f>B37-B36</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Estimativa central de Dublin</t>
-        </is>
-      </c>
-      <c r="B40" s="4">
-        <f>E33+B37*B39</f>
-        <v/>
+          <t>Aptos — portal (28 seções)</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>16720</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Teto: se as urnas ausentes tivessem 100% de comparecimento</t>
-        </is>
-      </c>
-      <c r="B41" s="4">
-        <f>E33+B37</f>
+          <t>Comparecimento % — portal</t>
+        </is>
+      </c>
+      <c r="B41" s="5">
+        <f>B37/B40</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Queda frente ao planejamento — piso (%)</t>
-        </is>
-      </c>
-      <c r="B42" s="5">
-        <f>B38/B36-1</f>
+          <t>Comparecimento das 5 urnas ausentes do PDF (portal − 23 urnas do PDF)</t>
+        </is>
+      </c>
+      <c r="B42" s="4">
+        <f>B37-E33</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Queda frente ao planejamento — estimativa central (%)</t>
-        </is>
-      </c>
-      <c r="B43" s="5">
-        <f>B40/B36-1</f>
+          <t>Aptos das 5 urnas ausentes (portal − 23 urnas do PDF)</t>
+        </is>
+      </c>
+      <c r="B43" s="4">
+        <f>B40-C33</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Queda frente ao planejamento — teto (%)</t>
+          <t>% comparecimento das 5 urnas ausentes</t>
         </is>
       </c>
       <c r="B44" s="5">
-        <f>B41/B36-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>A estimativa central é premissa, não dado: o comparecimento real das 5 urnas ausentes só sai do CSV/Resultados do TSE.</t>
+        <f>B42/B43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Estimativa anterior (mesma taxa das 23 urnas: 48,9%) — erro vs. real</t>
+        </is>
+      </c>
+      <c r="B45" s="4">
+        <f>(E33+B43*F33)-B37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Os dados do portal vêm das capturas de tela enviadas em 07/10/2026 (Dublin, 28/28 seções totalizadas). A diferença para o planejamento é de dado oficial, não de estimativa.</t>
         </is>
       </c>
     </row>
@@ -6502,7 +7342,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Soma dos municípios (aba "Por município")</t>
+          <t>Soma dos municípios (aba "Por município"; Dublin pelo portal)</t>
         </is>
       </c>
       <c r="B5" s="4">
@@ -6554,7 +7394,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>A diferença corresponde a seções sem ocorrência registrada, que o Anexo I não lista e o PDF não permite atribuir a município.</t>
+          <t>Dublin foi corrigido pelo portal (28 seções; o Anexo I omitia 5). Os demais ~19 mil eleitores / ~8,4 mil de comparecimento ainda não alocados são de seções omitidas do Anexo I em outros municípios.</t>
         </is>
       </c>
     </row>
@@ -6620,7 +7460,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dublin destacada em amarelo.</t>
+          <t>Dublin destacada em amarelo; conferidos 1:1 com o portal TSE: Genebra, Frankfurt, Edimburgo, Ciudad del Este (exatos) e Dublin (corrigida).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planilha do Exterior: corrige os 20 maiores municípios com o portal TSE
Valores lidos das capturas do portal (07/10/2026). 10 dos 20 diferiam do
Anexo I por seções omitidas (+7.157 eleitores, +3.487 comparecimento no
conjunto); os outros 10 conferem exatamente. Cobertura do total oficial
sobe para 98,5% (eleitores) e 98,2% (comparecimento). Coluna de fonte por linha.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bzScsAppuh4phNPSzsByq
</commit_message>
<xml_diff>
--- a/saidas/exterior_2026_t1_comparecimento_por_municipio.xlsx
+++ b/saidas/exterior_2026_t1_comparecimento_por_municipio.xlsx
@@ -489,7 +489,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="62" customWidth="1" min="9" max="9"/>
+    <col width="78" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -584,7 +584,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -601,13 +601,13 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>45891</v>
+        <v>47496</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>19510</v>
+        <v>20279</v>
       </c>
       <c r="G6" s="4">
         <f>E6-F6</f>
@@ -619,7 +619,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); corrigido vs Anexo I: +4 seção(ões); +1.605 eleitores; +769 comparecimento</t>
         </is>
       </c>
     </row>
@@ -628,21 +628,21 @@
         <v>3</v>
       </c>
       <c r="B7" t="n">
-        <v>30198</v>
+        <v>29416</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NAGÓIA</t>
+          <t>BOSTON</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>44536</v>
+        <v>53358</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>16317</v>
+        <v>16390</v>
       </c>
       <c r="G7" s="4">
         <f>E7-F7</f>
@@ -654,7 +654,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); corrigido vs Anexo I: +2 seção(ões); +796 eleitores; +196 comparecimento</t>
         </is>
       </c>
     </row>
@@ -663,21 +663,21 @@
         <v>4</v>
       </c>
       <c r="B8" t="n">
-        <v>29416</v>
+        <v>30198</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BOSTON</t>
+          <t>NAGÓIA</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>52562</v>
+        <v>44536</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>16194</v>
+        <v>16317</v>
       </c>
       <c r="G8" s="4">
         <f>E8-F8</f>
@@ -689,7 +689,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -706,13 +706,13 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>37052</v>
+        <v>37448</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>14586</v>
+        <v>14797</v>
       </c>
       <c r="G9" s="4">
         <f>E9-F9</f>
@@ -724,7 +724,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); corrigido vs Anexo I: +1 seção(ões); +396 eleitores; +211 comparecimento</t>
         </is>
       </c>
     </row>
@@ -741,13 +741,13 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>29640</v>
+        <v>30028</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>13166</v>
+        <v>13392</v>
       </c>
       <c r="G10" s="4">
         <f>E10-F10</f>
@@ -759,7 +759,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); corrigido vs Anexo I: +1 seção(ões); +388 eleitores; +226 comparecimento</t>
         </is>
       </c>
     </row>
@@ -776,13 +776,13 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>39654</v>
+        <v>40053</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>12166</v>
+        <v>12278</v>
       </c>
       <c r="G11" s="4">
         <f>E11-F11</f>
@@ -794,7 +794,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); corrigido vs Anexo I: +1 seção(ões); +399 eleitores; +112 comparecimento</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -873,21 +873,21 @@
         <v>10</v>
       </c>
       <c r="B14" t="n">
-        <v>99490</v>
+        <v>30635</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ORLANDO</t>
+          <t>TORONTO</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>26386</v>
+        <v>20953</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>8994</v>
+        <v>8999</v>
       </c>
       <c r="G14" s="4">
         <f>E14-F14</f>
@@ -899,7 +899,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); corrigido vs Anexo I: +1 seção(ões); +394 eleitores; +251 comparecimento</t>
         </is>
       </c>
     </row>
@@ -908,21 +908,21 @@
         <v>11</v>
       </c>
       <c r="B15" t="n">
-        <v>30635</v>
+        <v>99490</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>TORONTO</t>
+          <t>ORLANDO</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>20559</v>
+        <v>26386</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>8748</v>
+        <v>8994</v>
       </c>
       <c r="G15" s="4">
         <f>E15-F15</f>
@@ -934,7 +934,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Portal TSE (captura 07/10/2026) — substitui o Anexo I, que omitia 5 urnas</t>
+          <t>Portal TSE (07/10/2026); corrigido vs Anexo I: +5 seção(ões); +1.991 eleitores; +1.211 comparecimento</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -1091,13 +1091,13 @@
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>23065</v>
+        <v>23464</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>6738</v>
+        <v>6833</v>
       </c>
       <c r="G20" s="4">
         <f>E20-F20</f>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); corrigido vs Anexo I: +1 seção(ões); +399 eleitores; +95 comparecimento</t>
         </is>
       </c>
     </row>
@@ -1126,13 +1126,13 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>12357</v>
+        <v>12752</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>6235</v>
+        <v>6450</v>
       </c>
       <c r="G21" s="4">
         <f>E21-F21</f>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); corrigido vs Anexo I: +1 seção(ões); +395 eleitores; +215 comparecimento</t>
         </is>
       </c>
     </row>
@@ -1153,21 +1153,21 @@
         <v>18</v>
       </c>
       <c r="B22" t="n">
-        <v>30864</v>
+        <v>30155</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ZURIQUE</t>
+          <t>MONTREAL</t>
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>15099</v>
+        <v>10953</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>6001</v>
+        <v>6101</v>
       </c>
       <c r="G22" s="4">
         <f>E22-F22</f>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); corrigido vs Anexo I: +1 seção(ões); +394 eleitores; +201 comparecimento</t>
         </is>
       </c>
     </row>
@@ -1188,21 +1188,21 @@
         <v>19</v>
       </c>
       <c r="B23" t="n">
-        <v>39063</v>
+        <v>30864</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>VANCOUVER</t>
+          <t>ZURIQUE</t>
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>12082</v>
+        <v>15099</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>5912</v>
+        <v>6001</v>
       </c>
       <c r="G23" s="4">
         <f>E23-F23</f>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -1223,21 +1223,21 @@
         <v>20</v>
       </c>
       <c r="B24" t="n">
-        <v>30155</v>
+        <v>39063</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MONTREAL</t>
+          <t>VANCOUVER</t>
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>10559</v>
+        <v>12082</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>5900</v>
+        <v>5912</v>
       </c>
       <c r="G24" s="4">
         <f>E24-F24</f>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Anexo I (piso)</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Anexo I; confere com o portal</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Anexo I; confere com o portal</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Anexo I; confere com o portal</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Anexo I; confere com o portal</t>
+          <t>Portal TSE (07/10/2026); confere com o Anexo I</t>
         </is>
       </c>
     </row>
@@ -7342,7 +7342,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Soma dos municípios (aba "Por município"; Dublin pelo portal)</t>
+          <t>Soma dos municípios (aba "Por município"; 20 maiores pelo portal)</t>
         </is>
       </c>
       <c r="B5" s="4">
@@ -7394,7 +7394,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dublin foi corrigido pelo portal (28 seções; o Anexo I omitia 5). Os demais ~19 mil eleitores / ~8,4 mil de comparecimento ainda não alocados são de seções omitidas do Anexo I em outros municípios.</t>
+          <t>Os 20 maiores municípios (por comparecimento) foram conferidos/corrigidos com o portal TSE; 10 diferiam do Anexo I (seções omitidas). O que resta não alocado é de municípios menores, ainda só pelo Anexo I.</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dublin destacada em amarelo; conferidos 1:1 com o portal TSE: Genebra, Frankfurt, Edimburgo, Ciudad del Este (exatos) e Dublin (corrigida).</t>
+          <t>Dublin destacada em amarelo. Fonte por linha na coluna I: os 20 maiores (capturas do portal TSE de 07/10/2026) + Genebra, Frankfurt, Edimburgo e Ciudad del Este (conferidos, iguais ao Anexo I); demais municípios = Anexo I, piso.</t>
         </is>
       </c>
     </row>

</xml_diff>